<commit_message>
Add smart Excel column synonyms and safe fallbacks
</commit_message>
<xml_diff>
--- a/avs_internship_ready_for_upload.xlsx
+++ b/avs_internship_ready_for_upload.xlsx
@@ -433,7 +433,7 @@
         <v>IV</v>
       </c>
       <c r="E2" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F2" t="str">
         <v>IoT Application (ESP32)</v>
@@ -453,7 +453,7 @@
         <v>IV</v>
       </c>
       <c r="E3" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F3" t="str">
         <v>IoT Application (ESP32)</v>
@@ -473,7 +473,7 @@
         <v>IV</v>
       </c>
       <c r="E4" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F4" t="str">
         <v>IoT Application (ESP32)</v>
@@ -493,7 +493,7 @@
         <v>IV</v>
       </c>
       <c r="E5" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F5" t="str">
         <v>IoT Application (ESP32)</v>
@@ -513,7 +513,7 @@
         <v>IV</v>
       </c>
       <c r="E6" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F6" t="str">
         <v>IoT Application (ESP32)</v>
@@ -533,7 +533,7 @@
         <v>IV</v>
       </c>
       <c r="E7" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F7" t="str">
         <v>IoT Application (ESP32)</v>
@@ -553,7 +553,7 @@
         <v>IV</v>
       </c>
       <c r="E8" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F8" t="str">
         <v>IoT Application (ESP32)</v>
@@ -573,7 +573,7 @@
         <v>IV</v>
       </c>
       <c r="E9" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F9" t="str">
         <v>IoT Application (ESP32)</v>
@@ -593,7 +593,7 @@
         <v>IV</v>
       </c>
       <c r="E10" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F10" t="str">
         <v>IoT Application (ESP32)</v>
@@ -613,7 +613,7 @@
         <v>IV</v>
       </c>
       <c r="E11" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F11" t="str">
         <v>IoT Application (ESP32)</v>
@@ -633,7 +633,7 @@
         <v>IV</v>
       </c>
       <c r="E12" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F12" t="str">
         <v>IoT Application (ESP32)</v>
@@ -653,7 +653,7 @@
         <v>IV</v>
       </c>
       <c r="E13" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F13" t="str">
         <v>IoT Application (ESP32)</v>
@@ -673,7 +673,7 @@
         <v>IV</v>
       </c>
       <c r="E14" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F14" t="str">
         <v>IoT Application (ESP32)</v>
@@ -693,7 +693,7 @@
         <v>IV</v>
       </c>
       <c r="E15" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F15" t="str">
         <v>IoT Application (ESP32)</v>
@@ -713,7 +713,7 @@
         <v>IV</v>
       </c>
       <c r="E16" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F16" t="str">
         <v>IoT Application (ESP32)</v>
@@ -733,7 +733,7 @@
         <v>IV</v>
       </c>
       <c r="E17" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F17" t="str">
         <v>IoT Application (ESP32)</v>
@@ -753,7 +753,7 @@
         <v>IV</v>
       </c>
       <c r="E18" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F18" t="str">
         <v>IoT Application (ESP32)</v>
@@ -773,7 +773,7 @@
         <v>IV</v>
       </c>
       <c r="E19" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F19" t="str">
         <v>IoT Application (ESP32)</v>
@@ -793,7 +793,7 @@
         <v>IV</v>
       </c>
       <c r="E20" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F20" t="str">
         <v>IoT Application (ESP32)</v>
@@ -813,7 +813,7 @@
         <v>IV</v>
       </c>
       <c r="E21" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F21" t="str">
         <v>IoT Application (ESP32)</v>
@@ -833,7 +833,7 @@
         <v>IV</v>
       </c>
       <c r="E22" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F22" t="str">
         <v>IoT Application (ESP32)</v>
@@ -853,7 +853,7 @@
         <v>IV</v>
       </c>
       <c r="E23" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F23" t="str">
         <v>IoT Application (ESP32)</v>
@@ -873,7 +873,7 @@
         <v>IV</v>
       </c>
       <c r="E24" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F24" t="str">
         <v>IoT Application (ESP32)</v>
@@ -893,7 +893,7 @@
         <v>IV</v>
       </c>
       <c r="E25" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F25" t="str">
         <v>IoT Application (ESP32)</v>
@@ -913,7 +913,7 @@
         <v>IV</v>
       </c>
       <c r="E26" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F26" t="str">
         <v>IoT Application (ESP32)</v>
@@ -933,7 +933,7 @@
         <v>IV</v>
       </c>
       <c r="E27" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F27" t="str">
         <v>IoT Application (ESP32)</v>
@@ -953,7 +953,7 @@
         <v>IV</v>
       </c>
       <c r="E28" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F28" t="str">
         <v>IoT Application (ESP32)</v>
@@ -973,7 +973,7 @@
         <v>IV</v>
       </c>
       <c r="E29" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F29" t="str">
         <v>IoT Application (ESP32)</v>
@@ -993,7 +993,7 @@
         <v>IV</v>
       </c>
       <c r="E30" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F30" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1013,7 +1013,7 @@
         <v>IV</v>
       </c>
       <c r="E31" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F31" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1033,7 +1033,7 @@
         <v>IV</v>
       </c>
       <c r="E32" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F32" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1053,7 +1053,7 @@
         <v>IV</v>
       </c>
       <c r="E33" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F33" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1073,7 +1073,7 @@
         <v>IV</v>
       </c>
       <c r="E34" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F34" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1093,7 +1093,7 @@
         <v>IV</v>
       </c>
       <c r="E35" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F35" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1113,7 +1113,7 @@
         <v>IV</v>
       </c>
       <c r="E36" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F36" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1133,7 +1133,7 @@
         <v>IV</v>
       </c>
       <c r="E37" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F37" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1153,7 +1153,7 @@
         <v>IV</v>
       </c>
       <c r="E38" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F38" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1173,7 +1173,7 @@
         <v>IV</v>
       </c>
       <c r="E39" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F39" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1193,7 +1193,7 @@
         <v>IV</v>
       </c>
       <c r="E40" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F40" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1213,7 +1213,7 @@
         <v>IV</v>
       </c>
       <c r="E41" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F41" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1233,7 +1233,7 @@
         <v>IV</v>
       </c>
       <c r="E42" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F42" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1253,7 +1253,7 @@
         <v>IV</v>
       </c>
       <c r="E43" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F43" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1273,7 +1273,7 @@
         <v>IV</v>
       </c>
       <c r="E44" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F44" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1293,7 +1293,7 @@
         <v>IV</v>
       </c>
       <c r="E45" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F45" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1313,7 +1313,7 @@
         <v>IV</v>
       </c>
       <c r="E46" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F46" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1333,7 +1333,7 @@
         <v>IV</v>
       </c>
       <c r="E47" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F47" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1353,7 +1353,7 @@
         <v>IV</v>
       </c>
       <c r="E48" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F48" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1373,7 +1373,7 @@
         <v>IV</v>
       </c>
       <c r="E49" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F49" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1393,7 +1393,7 @@
         <v>IV</v>
       </c>
       <c r="E50" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F50" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1413,7 +1413,7 @@
         <v>IV</v>
       </c>
       <c r="E51" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F51" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1433,7 +1433,7 @@
         <v>IV</v>
       </c>
       <c r="E52" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F52" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1453,7 +1453,7 @@
         <v>IV</v>
       </c>
       <c r="E53" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F53" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1473,7 +1473,7 @@
         <v>IV</v>
       </c>
       <c r="E54" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F54" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1493,7 +1493,7 @@
         <v>IV</v>
       </c>
       <c r="E55" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F55" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1513,7 +1513,7 @@
         <v>IV</v>
       </c>
       <c r="E56" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F56" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1533,7 +1533,7 @@
         <v>IV</v>
       </c>
       <c r="E57" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F57" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1553,7 +1553,7 @@
         <v>IV</v>
       </c>
       <c r="E58" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F58" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1573,7 +1573,7 @@
         <v>IV</v>
       </c>
       <c r="E59" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F59" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1593,7 +1593,7 @@
         <v>IV</v>
       </c>
       <c r="E60" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F60" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1613,7 +1613,7 @@
         <v>IV</v>
       </c>
       <c r="E61" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F61" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1633,7 +1633,7 @@
         <v>IV</v>
       </c>
       <c r="E62" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F62" t="str">
         <v>IoT Application (ESP32)</v>
@@ -1653,7 +1653,7 @@
         <v>IV</v>
       </c>
       <c r="E63" t="str">
-        <v>SRITECH</v>
+        <v>SRI TECH</v>
       </c>
       <c r="F63" t="str">
         <v>IoT Application (ESP32)</v>

</xml_diff>